<commit_message>
fix tfa deaths averted computation
</commit_message>
<xml_diff>
--- a/scenarios/RTSL_Assessment_Results.xlsx
+++ b/scenarios/RTSL_Assessment_Results.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="294">
   <si>
     <t xml:space="preserve">Table 1. Program-attributable deaths averted (2017-2050) by intervention.</t>
   </si>
@@ -41,10 +41,10 @@
     <t xml:space="preserve">Observed RTSL program HTN control rates (2017–2024) maintained to 2050</t>
   </si>
   <si>
-    <t xml:space="preserve">368.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10.8</t>
+    <t xml:space="preserve">432.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.7</t>
   </si>
   <si>
     <t xml:space="preserve">TFA Elimination</t>
@@ -53,7 +53,10 @@
     <t xml:space="preserve">Industrial TFA elimination via best-practice policies enacted by 2024</t>
   </si>
   <si>
-    <t xml:space="preserve">0.0</t>
+    <t xml:space="preserve">19.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.6</t>
   </si>
   <si>
     <t xml:space="preserve">HTN Control + TFA Elimination</t>
@@ -62,7 +65,10 @@
     <t xml:space="preserve">Both interventions combined (multiplicative effects)</t>
   </si>
   <si>
-    <t xml:space="preserve">367.9</t>
+    <t xml:space="preserve">451.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.3</t>
   </si>
   <si>
     <t xml:space="preserve">Table 2. Deaths averted (thousands) by intervention and cause of death.</t>
@@ -83,25 +89,34 @@
     <t xml:space="preserve">Ischemic stroke</t>
   </si>
   <si>
-    <t xml:space="preserve">52.8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">85.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">135.8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">95.0</t>
+    <t xml:space="preserve">51.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">154.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">133.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">93.1</t>
   </si>
   <si>
     <t xml:space="preserve">–</t>
   </si>
   <si>
-    <t xml:space="preserve">135.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">95.1</t>
+    <t xml:space="preserve">20.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">51.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">154.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">152.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92.7</t>
   </si>
   <si>
     <t xml:space="preserve">Table 3. Deaths averted by age group and intervention.</t>
@@ -1287,21 +1302,21 @@
         <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D6" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -1324,24 +1339,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -1349,16 +1364,16 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5">
@@ -1366,33 +1381,33 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D5" t="s">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="E5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="D6" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="E6" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1417,306 +1432,306 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="E4" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="F4" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="G4" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="D5" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="E5" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F5" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="G5" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D6" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="E6" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="F6" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="G6" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="D7" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E7" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F7" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="G7" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
       </c>
       <c r="C8" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="D8" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="E8" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F8" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="G8" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="D9" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="E9" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="F9" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="G9" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B10" t="s">
         <v>5</v>
       </c>
       <c r="C10" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="D10" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="E10" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="F10" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="G10" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B11" t="s">
         <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D11" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="E11" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F11" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="G11" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C12" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="D12" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E12" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="F12" t="s">
+        <v>76</v>
+      </c>
+      <c r="G12" t="s">
         <v>71</v>
-      </c>
-      <c r="G12" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B13" t="s">
         <v>5</v>
       </c>
       <c r="C13" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="D13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E13" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F13" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="G13" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B14" t="s">
         <v>9</v>
       </c>
       <c r="C14" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D14" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E14" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F14" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="G14" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B15" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C15" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="D15" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E15" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="F15" t="s">
+        <v>87</v>
+      </c>
+      <c r="G15" t="s">
         <v>82</v>
-      </c>
-      <c r="G15" t="s">
-        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1741,651 +1756,651 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B4" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="C4" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D4" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="E4" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="F4" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="G4" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B5" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="C5" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="D5" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E5" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="F5" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="G5" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B6" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="C6" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D6" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="E6" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="F6" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="G6" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B7" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C7" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="D7" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="E7" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="F7" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="G7" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B8" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="C8" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D8" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="E8" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="F8" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="G8" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B9" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="C9" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="D9" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="E9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="F9" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="G9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B10" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="C10" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="D10" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="E10" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="F10" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="G10" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B11" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="C11" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="D11" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="E11" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="F11" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="G11" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B12" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C12" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D12" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="E12" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="F12" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="G12" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B13" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C13" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="D13" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="E13" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="F13" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="G13" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B14" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="C14" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="D14" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="E14" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="F14" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="G14" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B15" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="C15" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D15" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E15" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="F15" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="G15" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B16" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="C16" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="D16" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="E16" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="F16" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="G16" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B17" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C17" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="D17" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="E17" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="F17" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="G17" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B18" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C18" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="D18" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="E18" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="F18" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="G18" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="B19" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="C19" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="D19" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="E19" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="F19" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="G19" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="B20" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="C20" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="D20" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="E20" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="F20" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="G20" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="B21" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="C21" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="D21" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="E21" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="F21" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="G21" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B22" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="C22" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="D22" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="E22" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="F22" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="G22" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B23" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="C23" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="D23" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="E23" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="F23" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="G23" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B24" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="C24" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="D24" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="E24" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="F24" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="G24" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B25" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="C25" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="D25" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="E25" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="F25" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="G25" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B26" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="C26" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="D26" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="E26" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="F26" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="G26" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B27" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="C27" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="D27" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="E27" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="F27" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="G27" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="B28" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C28" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="D28" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="E28" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="F28" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="G28" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="B29" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="C29" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="D29" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="E29" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="F29" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="G29" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="B30" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="C30" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="D30" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="E30" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="F30" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="G30" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -2409,127 +2424,127 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B4" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="C4" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="D4" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="E4" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="F4" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B5" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="C5" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="D5" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="E5" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="F5" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="B6" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C6" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D6" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="E6" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="F6" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B7" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="C7" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="D7" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="E7" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="F7" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="B8" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C8" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D8" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="E8" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="F8" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
     </row>
   </sheetData>
@@ -2549,55 +2564,55 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B4" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B5" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="B6" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B7" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="B8" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
     </row>
   </sheetData>
@@ -2619,399 +2634,399 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>100</v>
+        <v>203</v>
       </c>
       <c r="B4" t="n">
-        <v>11203.4256500206</v>
+        <v>14440.2677629494</v>
       </c>
       <c r="C4" t="n">
-        <v>35019.8876997908</v>
+        <v>30802.4430895314</v>
       </c>
       <c r="D4" t="n">
-        <v>0.319916092994426</v>
+        <v>0.468802676494745</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>198</v>
+        <v>105</v>
       </c>
       <c r="B5" t="n">
-        <v>11201.3886264814</v>
+        <v>13330.2018703025</v>
       </c>
       <c r="C5" t="n">
-        <v>26203.5711380414</v>
+        <v>38194.3629714381</v>
       </c>
       <c r="D5" t="n">
-        <v>0.427475650836754</v>
+        <v>0.349009666171704</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>118</v>
+        <v>184</v>
       </c>
       <c r="B6" t="n">
-        <v>6803.05148166196</v>
+        <v>8918.14153710502</v>
       </c>
       <c r="C6" t="n">
-        <v>22873.0273559241</v>
+        <v>18277.8980036463</v>
       </c>
       <c r="D6" t="n">
-        <v>0.297426806508845</v>
+        <v>0.487919427897338</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>142</v>
+        <v>123</v>
       </c>
       <c r="B7" t="n">
-        <v>6387.27058607015</v>
+        <v>8378.85310090075</v>
       </c>
       <c r="C7" t="n">
-        <v>18340.8411139692</v>
+        <v>25718.0741912707</v>
       </c>
       <c r="D7" t="n">
-        <v>0.348253962093665</v>
+        <v>0.325796287800768</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="B8" t="n">
-        <v>5812.01295917907</v>
+        <v>7989.61156281484</v>
       </c>
       <c r="C8" t="n">
-        <v>13642.5516097569</v>
+        <v>16674.0127135217</v>
       </c>
       <c r="D8" t="n">
-        <v>0.426020961872149</v>
+        <v>0.479165495438043</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>124</v>
+        <v>221</v>
       </c>
       <c r="B9" t="n">
-        <v>5650.23251802824</v>
+        <v>7621.13796525535</v>
       </c>
       <c r="C9" t="n">
-        <v>22717.1062838141</v>
+        <v>12121.4324365247</v>
       </c>
       <c r="D9" t="n">
-        <v>0.248721489763598</v>
+        <v>0.628732454284123</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="B10" t="n">
-        <v>5585.19683319401</v>
+        <v>7588.68043401262</v>
       </c>
       <c r="C10" t="n">
-        <v>13349.3585584744</v>
+        <v>14613.6540347195</v>
       </c>
       <c r="D10" t="n">
-        <v>0.418386906661401</v>
+        <v>0.519286991192157</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>112</v>
+        <v>147</v>
       </c>
       <c r="B11" t="n">
-        <v>4961.74186449536</v>
+        <v>7555.33407000994</v>
       </c>
       <c r="C11" t="n">
-        <v>24768.195550673</v>
+        <v>20177.490532851</v>
       </c>
       <c r="D11" t="n">
-        <v>0.200327143507252</v>
+        <v>0.37444369297109</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>130</v>
+        <v>215</v>
       </c>
       <c r="B12" t="n">
-        <v>4766.62090515151</v>
+        <v>6588.33827778888</v>
       </c>
       <c r="C12" t="n">
-        <v>21096.7122362352</v>
+        <v>17850.3652089038</v>
       </c>
       <c r="D12" t="n">
-        <v>0.225941409816667</v>
+        <v>0.369087029911445</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>106</v>
+        <v>246</v>
       </c>
       <c r="B13" t="n">
-        <v>4444.57204246794</v>
+        <v>6103.41191869952</v>
       </c>
       <c r="C13" t="n">
-        <v>24896.9402541938</v>
+        <v>12141.3286072061</v>
       </c>
       <c r="D13" t="n">
-        <v>0.178518805808648</v>
+        <v>0.502697201941887</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>241</v>
+        <v>135</v>
       </c>
       <c r="B14" t="n">
-        <v>3845.3773726513</v>
+        <v>6063.10177818698</v>
       </c>
       <c r="C14" t="n">
-        <v>9030.18919696993</v>
+        <v>23363.5215872276</v>
       </c>
       <c r="D14" t="n">
-        <v>0.425835748152609</v>
+        <v>0.259511467719043</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>204</v>
+        <v>129</v>
       </c>
       <c r="B15" t="n">
-        <v>3828.05416387019</v>
+        <v>6012.41496979775</v>
       </c>
       <c r="C15" t="n">
-        <v>14724.236717965</v>
+        <v>23568.2845691785</v>
       </c>
       <c r="D15" t="n">
-        <v>0.259983198938902</v>
+        <v>0.255106176783884</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>210</v>
+        <v>117</v>
       </c>
       <c r="B16" t="n">
-        <v>3781.88518175636</v>
+        <v>5781.72234934512</v>
       </c>
       <c r="C16" t="n">
-        <v>12510.5042474009</v>
+        <v>26509.667884509</v>
       </c>
       <c r="D16" t="n">
-        <v>0.302296782525137</v>
+        <v>0.21809863384685</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="B17" t="n">
-        <v>3472.17825912695</v>
+        <v>5599.31276845992</v>
       </c>
       <c r="C17" t="n">
-        <v>7062.41670896377</v>
+        <v>9653.39191983159</v>
       </c>
       <c r="D17" t="n">
-        <v>0.491641657836473</v>
+        <v>0.580035785862676</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>148</v>
+        <v>196</v>
       </c>
       <c r="B18" t="n">
-        <v>3455.69932592117</v>
+        <v>5469.07287186178</v>
       </c>
       <c r="C18" t="n">
-        <v>14891.5238949211</v>
+        <v>8312.59427168696</v>
       </c>
       <c r="D18" t="n">
-        <v>0.232058139268055</v>
+        <v>0.657926117059468</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B19" t="n">
-        <v>3323.54652694761</v>
+        <v>5120.07838971769</v>
       </c>
       <c r="C19" t="n">
-        <v>13384.068850399</v>
+        <v>18807.6971561717</v>
       </c>
       <c r="D19" t="n">
-        <v>0.248321087114591</v>
+        <v>0.272233136635632</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>136</v>
+        <v>209</v>
       </c>
       <c r="B20" t="n">
-        <v>3314.18358769326</v>
+        <v>4745.57827539977</v>
       </c>
       <c r="C20" t="n">
-        <v>18955.8881973081</v>
+        <v>17147.4279464284</v>
       </c>
       <c r="D20" t="n">
-        <v>0.174836628766564</v>
+        <v>0.276751609059142</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>185</v>
+        <v>111</v>
       </c>
       <c r="B21" t="n">
-        <v>3297.52534319387</v>
+        <v>4646.55804753599</v>
       </c>
       <c r="C21" t="n">
-        <v>8371.30367918487</v>
+        <v>25603.9439523479</v>
       </c>
       <c r="D21" t="n">
-        <v>0.393908221415157</v>
+        <v>0.181478215082169</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>87</v>
+        <v>141</v>
       </c>
       <c r="B22" t="n">
-        <v>2821.85272567379</v>
+        <v>3785.58349779321</v>
       </c>
       <c r="C22" t="n">
-        <v>18307.6035169044</v>
+        <v>20206.2821111541</v>
       </c>
       <c r="D22" t="n">
-        <v>0.15413556029156</v>
+        <v>0.187346859603803</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>93</v>
+        <v>159</v>
       </c>
       <c r="B23" t="n">
-        <v>2227.50078085901</v>
+        <v>3707.86280291735</v>
       </c>
       <c r="C23" t="n">
-        <v>11293.8282353853</v>
+        <v>14318.0103931896</v>
       </c>
       <c r="D23" t="n">
-        <v>0.197231685698912</v>
+        <v>0.258964947020921</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>216</v>
+        <v>98</v>
       </c>
       <c r="B24" t="n">
-        <v>1990.61652531912</v>
+        <v>3115.97660093583</v>
       </c>
       <c r="C24" t="n">
-        <v>4529.80859961483</v>
+        <v>13502.415275421</v>
       </c>
       <c r="D24" t="n">
-        <v>0.439448263992518</v>
+        <v>0.230771794332824</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>191</v>
+        <v>92</v>
       </c>
       <c r="B25" t="n">
-        <v>1117.31095319002</v>
+        <v>3071.79487815121</v>
       </c>
       <c r="C25" t="n">
-        <v>2513.93431933336</v>
+        <v>19277.1558045535</v>
       </c>
       <c r="D25" t="n">
-        <v>0.444447153848598</v>
+        <v>0.159348967726122</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
       <c r="B26" t="n">
-        <v>1115.44864689192</v>
+        <v>2206.48162616365</v>
       </c>
       <c r="C26" t="n">
-        <v>4769.84621581293</v>
+        <v>3810.53722191088</v>
       </c>
       <c r="D26" t="n">
-        <v>0.23385421592713</v>
+        <v>0.579047388246522</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B27" t="n">
-        <v>485.667180670922</v>
+        <v>1625.2220002968</v>
       </c>
       <c r="C27" t="n">
-        <v>1528.84467461446</v>
+        <v>5236.97631157674</v>
       </c>
       <c r="D27" t="n">
-        <v>0.317669406667093</v>
+        <v>0.310335946470509</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="B28" t="n">
-        <v>446.219798315781</v>
+        <v>1571.45145193124</v>
       </c>
       <c r="C28" t="n">
-        <v>2273.93354788419</v>
+        <v>6889.40389023085</v>
       </c>
       <c r="D28" t="n">
-        <v>0.19623255865633</v>
+        <v>0.2280968683168</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="B29" t="n">
-        <v>138.063952426151</v>
+        <v>1278.92434327408</v>
       </c>
       <c r="C29" t="n">
-        <v>339.381465742158</v>
+        <v>5302.42122231</v>
       </c>
       <c r="D29" t="n">
-        <v>0.406810525507731</v>
+        <v>0.241196293099649</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="B30" t="n">
-        <v>127.459497263519</v>
+        <v>1037.45840882131</v>
       </c>
       <c r="C30" t="n">
-        <v>472.778664231038</v>
+        <v>3241.68609164268</v>
       </c>
       <c r="D30" t="n">
-        <v>0.269596551000939</v>
+        <v>0.320036665948612</v>
       </c>
     </row>
   </sheetData>

</xml_diff>